<commit_message>
data(tg-whatsapp-rag): aplicar las instrucciones de carga al catálogo
Aplica el contenido preparado en el commit anterior. La hoja Instrucciones pasa
de 41 a 122 filas, dividida en cotizar (lo que ya estaba) y cargar (nuevo).

Solo cambiaron sheet1.xml y sharedStrings.xml; las 6 hojas de datos quedaron
byte-idénticas. Estilos, validaciones, definedNames y el hidden de _listas
verificados intactos. ZIP validado: 13/13 entradas con CRC y tamaño correctos.

Visor sobre el archivo nuevo: los 7 chunks sin cambios. 56 tests en verde.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
   <si>
     <t xml:space="preserve">CÓMO SE COTIZA — leer antes de tocar nada</t>
   </si>
@@ -507,6 +507,225 @@
   </si>
   <si>
     <t xml:space="preserve">Colecciones — desplegable de Productos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÓMO USAR ESTE ARCHIVO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La primera parte explica cómo COTIZAR (leer). La segunda, cómo CARGAR cosas nuevas (escribir).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">═══ PARTE 1: CÓMO COTIZAR ═══</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODO "pliego" (stickers y etiquetas en papel autoadhesivo u OPP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Piezas por pliego: la columna "Piezas por pliego" del producto ya trae el número.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODO "m2" (vinilos, lonas, carteles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿CUÁL DE LOS DOS MODOS?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo decide la columna "Unidad" del MATERIAL, no el producto. Si empieza con "pliego" → modo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pliego. Si es "m2" → modo m2. El producto no dice el modo en ningún lado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">═══ PARTE 2: CÓMO CARGAR COSAS NUEVAS ═══</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAS HOJAS Y PARA QUÉ SIRVEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colecciones — las familias de productos. Su descripción encabeza el bloque que lee el bot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productos   — lo que se ofrece. La cantidad NO va acá: la pide el cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales  — precios y tramos. Un material sin escala por volumen = un solo tramo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parámetros  — mínimo por trabajo, redondeo, moneda.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Casos de prueba — NO se usa para cotizar. Verifica que el bot calcula bien.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_listas     — hoja OCULTA. Alimenta los desplegables. Ver abajo, hay que tocarla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL ORDEN IMPORTA: colección → material → producto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las columnas Colección y Material de la hoja Productos son DESPLEGABLES. Solo ofrecen valores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">que ya existen. Si cargás el producto primero, el desplegable no va a tener qué ofrecerte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJEMPLO COMPLETO: producto nuevo, material nuevo, colección nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedido: "agregar imanes de heladera 8x5 cm, se hacen en imán flexible, $18.000 el m2, mínimo 0,3 m2".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASO 1 — Colección nueva. En la hoja Colecciones, primera fila libre:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Colección:   Imanes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Descripción: Imanes flexibles impresos full color, cortados con forma. Para heladera,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                pizarras y superficies metálicas. Se cotizan por metro cuadrado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   La descripción es lo que lee el bot: que se entienda sola, sin nombrar otras colecciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASO 2 — Material nuevo. En la hoja Materiales, primera fila libre:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Material: Imán flexible | Unidad: m2 | Desde: 1 | Hasta: (vacío)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Precio por unidad: 18000 | Mínimo facturable: 0,3 | Nota: confirmado el 26/08/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASO 3 — Registrar los dos en _listas (la hoja oculta). SIN ESTE PASO LOS DESPLEGABLES NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   LOS OFRECEN. Mostrar la hoja (clic derecho en las pestañas → Mostrar) y agregar:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   columna A → el material nuevo   ·   columna B → la colección nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Van en la primera fila libre de cada columna, sin dejar huecos en el medio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASO 4 — Producto. En la hoja Productos, primera fila libre:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Colección: Imanes (ya aparece en el desplegable) | Producto: Imán 8x5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Descripción: Imán flexible impreso full color, cortado con forma.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Material: Imán flexible | Ancho: 8 | Alto: 5 | Piezas por pliego: (vacío, es modo m2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUÉ COLUMNAS SON OBLIGATORIAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depende del modo del material, y es al revés en cada uno:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Modo pliego → el PRODUCTO necesita 'Piezas por pliego'. El material NO lleva mínimo facturable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Modo m2     → el MATERIAL necesita 'Mínimo facturable'. El producto deja 'Piezas por pliego' vacío.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una columna vacía no es un error: es lo que hace que el bot no vea datos que no corresponden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÓMO SE ESCRIBE UNA ESCALA DE PRECIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un material = una o más filas en Materiales, todas con el MISMO nombre en la columna Material.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Precio fijo, sin descuento por volumen → UNA fila: Desde 1, Hasta vacío.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Con descuento por volumen → una fila por tramo. Desde/Hasta sin huecos ni superposiciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   El último tramo va con Hasta VACÍO: significa 'de acá en adelante'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Ejemplo de escala: 1 a 1 → 2500 · 2 a 10 → 2200 · 11 a 50 → 2000 · 101 a (vacío) → 1710</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE DÓNDE SALE "PIEZAS POR PLIEGO"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es geometría, no un dato que se inventa. Sobre el pliego A3, con estas áreas útiles:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Troquelado o medio corte: 28 x 44 cm, con 0,3 cm de separación entre piezas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Solo impresión:           31 x 46 cm, sin separación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fórmula: (columnas que entran a lo ancho) × (filas que entran a lo alto), redondeando cada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">división HACIA ABAJO. Se prueban las DOS orientaciones y se toma la que rinde más.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Ejemplo: pieza de 12x8 troquelada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Acostada (12 de ancho): 28,3÷12,3 = 2 columnas × 44,3÷8,3 = 5 filas = 10 piezas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Parada   (8 de ancho):  28,3÷8,3 = 3 columnas × 44,3÷12,3 = 3 filas = 9 piezas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Se toma 10. (Se suma la separación al área y a la pieza antes de dividir.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LÍMITES DE CRECIMIENTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los desplegables y la validación cubren un rango fijo. Hoy hay lugar para:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Productos: hasta la fila 72 · Materiales en _listas: hasta A42 · Colecciones: hasta B35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasado eso el desplegable deja de funcionar SIN AVISAR. Si se llega al tope, hay que extender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">el rango (Datos → Validación) y el nombre definido, o avisar para que lo hagamos nosotros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRORES QUE ROMPEN EN SILENCIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Escribir el material a mano con una letra distinta a la de Materiales: el producto queda sin precio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Poner "por pliego" o "metro cuadrado" en Unidad: solo valen "pliego A3" y "m2".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Dejar 'Piezas por pliego' vacío en un producto de modo pliego: no se puede cotizar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Tramos superpuestos (1-10 y 5-20): se aplica el primero que coincide, y puede no ser el que querías.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Cargar un producto en una colección que no existe en la hoja Colecciones: queda sin descripción.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESPUÉS DE EDITAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guardar el archivo y volver a cargarlo en el visor de chunks para ver qué va a leer el bot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los cambios NO llegan al bot hasta que se ingesta desde ahí.</t>
   </si>
 </sst>
 </file>
@@ -692,7 +911,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2"/>
@@ -709,150 +928,479 @@
     <row r="5"/>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="s">
+    <row r="14">
+      <c r="A14" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="11" t="s">
+    <row r="15">
+      <c r="A15" s="11" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="12" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="11" t="s">
-        <v>11</v>
+      <c r="A17" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="s">
+    <row r="24">
+      <c r="A24" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="s">
+    <row r="25">
+      <c r="A25" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="s">
+    <row r="26">
+      <c r="A26" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="12" t="s">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="s">
+    <row r="29">
+      <c r="A29" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="12" t="s">
+    <row r="30">
+      <c r="A30" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="10" t="s">
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="10" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="11" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="41">
       <c r="A41" s="11" t="s">
-        <v>30</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="11" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76">
+      <c r="A76" s="11" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="80"/>
+    <row r="81">
+      <c r="A81" s="10" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="86"/>
+    <row r="87">
+      <c r="A87" s="10" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="92"/>
+    <row r="93">
+      <c r="A93" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="94"/>
+    <row r="95">
+      <c r="A95" s="10" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="101"/>
+    <row r="102">
+      <c r="A102" s="12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="106"/>
+    <row r="107">
+      <c r="A107" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="11" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="112"/>
+    <row r="113">
+      <c r="A113" s="10" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="119"/>
+    <row r="120">
+      <c r="A120" s="10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(tg-whatsapp-rag): Excel migrado al motor de medida libre
Geometría como dato en Materiales (28x44/0,3 troquelado · 31x46/0 solo
impresión), rinde vaciado en los 14 productos pliego (14/14 validados
contra el cálculo antes de borrar), Instrucciones con la fórmula de
encaje en la PARTE 1, y 7 casos de prueba nuevos (medida libre, rotación,
no-entra, mínimo por trabajo, redondeo).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="272">
   <si>
     <t xml:space="preserve">CÓMO USAR ESTE ARCHIVO</t>
   </si>
@@ -732,6 +732,120 @@
   </si>
   <si>
     <t xml:space="preserve">(Para otras unidades — una bobina, una plancha — es cuántas piezas rinde: dato del taller.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área útil ancho (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área útil alto (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separación (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada producto dice de qué material se hace. Las medidas del catálogo son REFERENCIAS: se cotiza CUALQUIER medida que pida el cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Rinde: cuántas piezas entran en una unidad de cobro. Se calcula con la geometría del</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   MATERIAL (hoja Materiales: 'Área útil ancho/alto (cm)' y 'Separación (cm)'):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   columnas × filas que entran = floor((útil + sep) ÷ (pieza + sep)) en cada eje,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   probando las DOS orientaciones y tomando la que rinde más. Vale CUALQUIER medida.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Ejemplo: pieza de 12x8 troquelada (área útil 28x44, separación 0,3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Acostada: 28,3÷12,3 = 2 columnas × 44,3÷8,3 = 5 filas = 10. Parada: 3 × 3 = 9. → 10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Si el rinde da 0 (la pieza no entra en ninguna orientación), NO cotizar: derivar a consulta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. m2 de una pieza = (ancho × alto) ÷ 10.000. Las medidas están en centímetros. Vale CUALQUIER medida.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   (Material de PLIEGO: cargar también 'Área útil ancho/alto (cm)' y 'Separación (cm)',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   una sola vez, en la primera fila del material.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Modo pliego → el MATERIAL necesita 'Área útil ancho/alto (cm)' y 'Separación (cm)';</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 no lleva mínimo facturable. El producto deja el rinde VACÍO: se calcula.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 'Piezas por unidad de cobro' se carga SOLO para unidades no geométricas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya NO se carga a mano para los pliegos. La geometría se declara UNA vez por material en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la hoja Materiales ('Área útil ancho/alto (cm)' y 'Separación (cm)') y el rinde se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">calcula solo, con la fórmula de la PARTE 1: el visor lo calcula para las medidas de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">referencia y el bot para cualquier otra medida que pida el cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Troquelado o medio corte: área útil 28 x 44 cm, separación 0,3 cm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Solo impresión:           área útil 31 x 46 cm, separación 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La columna 'Piezas por unidad de cobro' queda SOLO para unidades no geométricas — una</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bobina, una plancha — donde el rinde es dato del taller, no geometría. Si se carga,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manda sobre el cálculo, y el visor avisa si no coincide con la geometría.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Material de modo pliego sin geometría: no hay de dónde calcular el rinde. El visor lo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  avisa al cargar el archivo; hasta cargarla, el bot no puede cotizar ese material.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Rinde cargado a mano Y geometría que no coinciden: gana el dato cargado y el visor avisa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Pieza más grande que el área útil: rinde 0. Se deriva a consulta, nunca se inventa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">500 stickers 2x2 cm (medida libre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 etiquetas 5x8 cm (medida libre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80 etiquetas 20x6 cm (gana la orientación rotada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300 etiquetas 4x4 cm solo impresión (sin separación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 stickers 30x45 cm (no entra en el pliego)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derivar a consulta: no entra en el pliego</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 stickers 3x3 cm (activa el mínimo por trabajo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 lona de 90x60 cm (activa el redondeo)</t>
   </si>
 </sst>
 </file>
@@ -1135,7 +1249,7 @@
     <tabColor rgb="FF3B424F"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A147"/>
+  <dimension ref="A1:A156"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="105"/>
@@ -1151,584 +1265,637 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
+    <row r="3" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+    <row r="6" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="9" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
     <row r="12" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>6</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>7</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>8</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="22" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="23" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="24" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="26" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+    <row r="27" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+    <row r="31" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="32" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+    <row r="33" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+    <row r="34" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+    <row r="35" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="31" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+    <row r="37" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="38" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
+    <row r="45" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="40" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+    <row r="46" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="46" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
+    <row r="47" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="55" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="57" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A57" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
     <row r="59" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
-        <v>39</v>
+      <c r="A59" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="60" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="61" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="62" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
-        <v>41</v>
+      <c r="A62" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="63" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="s">
-        <v>42</v>
+      <c r="A63" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="64" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="66" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="68" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="69" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="70" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A70" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="72" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="73" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="75" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A75" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
     <row r="77" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>53</v>
+        <v>247</v>
       </c>
     </row>
     <row r="78" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="4" t="s">
-        <v>54</v>
+      <c r="A78" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="79" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A79" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="82" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2" t="s">
-        <v>57</v>
+      <c r="A82" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="83" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="84" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
+      <c r="A84" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="86" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A86" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="88" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="2" t="s">
-        <v>62</v>
+      <c r="A88" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="89" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="91" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>65</v>
+        <v>248</v>
       </c>
     </row>
     <row r="92" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A92" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
     <row r="94" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A94" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
     <row r="96" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="s">
-        <v>68</v>
+      <c r="A96" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="97" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="99" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="100" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="101" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="102" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="104" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="105" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="4" t="s">
-        <v>75</v>
+      <c r="A105" s="2" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="106" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="4" t="s">
-        <v>76</v>
+      <c r="A106" s="2" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="107" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A107" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
     <row r="109" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>78</v>
+        <v>255</v>
       </c>
     </row>
     <row r="110" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>79</v>
+        <v>256</v>
       </c>
     </row>
     <row r="111" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>80</v>
+        <v>257</v>
       </c>
     </row>
     <row r="112" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>81</v>
+        <v>258</v>
       </c>
     </row>
     <row r="113" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="3" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A113" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
     <row r="115" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="2" t="s">
-        <v>214</v>
-      </c>
-    </row>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="117" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>215</v>
+        <v>79</v>
       </c>
     </row>
     <row r="118" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
     <row r="120" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="2" t="s">
-        <v>217</v>
+      <c r="A120" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="121" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="4" t="s">
-        <v>218</v>
+      <c r="A121" s="2" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="122" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="123" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="4" t="s">
-        <v>219</v>
+      <c r="A123" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="124" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="4" t="s">
-        <v>220</v>
+      <c r="A124" s="2" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="125" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="4" t="s">
-        <v>221</v>
+      <c r="A125" s="2" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="126" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="3" t="s">
-        <v>222</v>
+      <c r="A126" s="2" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="127" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="128" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="2" t="s">
+      <c r="A128" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="131" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="2" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="129" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="2" t="s">
+    <row r="135" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="136" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="2" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="130" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="2" t="s">
+    <row r="137" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="131" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="133" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="4" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="135" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="4" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="136" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="138" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>83</v>
+        <v>226</v>
       </c>
     </row>
     <row r="139" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="140" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="2" t="s">
-        <v>231</v>
+      <c r="A140" s="4" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="141" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
+      <c r="A141" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="143" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="2" t="s">
-        <v>87</v>
+      <c r="A143" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="144" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="3" t="s">
-        <v>88</v>
+      <c r="A144" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="145" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="146" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>89</v>
+        <v>230</v>
       </c>
     </row>
     <row r="147" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="156" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1867,9 +2034,6 @@
       <c r="F2" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="9" t="n">
-        <v>104</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
@@ -1890,9 +2054,6 @@
       <c r="F3" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="9" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
@@ -1913,9 +2074,6 @@
       <c r="F4" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="9" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
@@ -1936,9 +2094,6 @@
       <c r="F5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="9" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
@@ -1959,9 +2114,6 @@
       <c r="F6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="9" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
@@ -1982,9 +2134,6 @@
       <c r="F7" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="9" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
@@ -2005,9 +2154,6 @@
       <c r="F8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="9" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
@@ -2028,9 +2174,6 @@
       <c r="F9" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="G9" s="9" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
@@ -2051,9 +2194,6 @@
       <c r="F10" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="9" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
@@ -2074,9 +2214,6 @@
       <c r="F11" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="G11" s="9" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
@@ -2097,9 +2234,6 @@
       <c r="F12" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="9" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
@@ -2120,9 +2254,6 @@
       <c r="F13" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G13" s="9" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
@@ -2143,9 +2274,6 @@
       <c r="F14" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G14" s="9" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
@@ -2165,9 +2293,6 @@
       </c>
       <c r="F15" s="9" t="n">
         <v>10</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2537,7 +2662,7 @@
     <tabColor rgb="FFBF8F00"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47"/>
@@ -2546,6 +2671,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2570,6 +2696,15 @@
       <c r="G1" s="5" t="s">
         <v>165</v>
       </c>
+      <c r="H1" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
@@ -2588,6 +2723,15 @@
         <v>2500</v>
       </c>
       <c r="G2" s="11"/>
+      <c r="H2" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
@@ -2672,6 +2816,15 @@
         <v>1800</v>
       </c>
       <c r="G7" s="11"/>
+      <c r="H7" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
@@ -2705,6 +2858,15 @@
         <v>2400</v>
       </c>
       <c r="G9" s="11"/>
+      <c r="H9" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
@@ -2756,6 +2918,15 @@
         <v>2800</v>
       </c>
       <c r="G12" s="11"/>
+      <c r="H12" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
@@ -2807,6 +2978,15 @@
         <v>2600</v>
       </c>
       <c r="G15" s="11"/>
+      <c r="H15" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -2858,6 +3038,15 @@
         <v>3000</v>
       </c>
       <c r="G18" s="11"/>
+      <c r="H18" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
@@ -3068,7 +3257,7 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -3941,6 +4130,164 @@
       </c>
       <c r="G40" s="14" t="n">
         <v>64000</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>228</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>8800</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>300</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>104</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>8600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(tg-whatsapp-rag): columna Material base en Colecciones + dropdown (script quirúrgico)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="273">
   <si>
     <t xml:space="preserve">CÓMO USAR ESTE ARCHIVO</t>
   </si>
@@ -846,6 +846,9 @@
   </si>
   <si>
     <t xml:space="preserve">1 lona de 90x60 cm (activa el redondeo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material base</t>
   </si>
 </sst>
 </file>
@@ -1916,11 +1919,12 @@
     <tabColor rgb="FF7030A0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="104"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1930,6 +1934,9 @@
       <c r="B1" s="5" t="s">
         <v>92</v>
       </c>
+      <c r="C1" s="5" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
@@ -1938,6 +1945,9 @@
       <c r="B2" s="7" t="s">
         <v>94</v>
       </c>
+      <c r="C2" s="6" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
@@ -1946,6 +1956,9 @@
       <c r="B3" s="7" t="s">
         <v>96</v>
       </c>
+      <c r="C3" s="6" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
@@ -1954,6 +1967,9 @@
       <c r="B4" s="7" t="s">
         <v>98</v>
       </c>
+      <c r="C4" s="6" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
@@ -1962,8 +1978,17 @@
       <c r="B5" s="7" t="s">
         <v>100</v>
       </c>
+      <c r="C5" s="6" t="s">
+        <v>155</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" error="Elegí un material de la lista desplegable. Si necesitás uno nuevo, agregalo primero en la hoja Materiales." errorStyle="stop" errorTitle="Ese material no existe" operator="between" prompt="El material que se cotiza cuando el cliente no pide una opción especial. Sale de la hoja Materiales." promptTitle="Material base" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C35" type="list">
+      <formula1>Materiales_lista</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>